<commit_message>
Removed temporary Excel files
</commit_message>
<xml_diff>
--- a/info/defences/defencesDatabase.xlsx
+++ b/info/defences/defencesDatabase.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ayuu/Developer/arxstudios/clashex/info/defences/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{992362BB-18B5-1B45-BADB-474F5A4CB767}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05282831-63B6-FF48-967E-0FD70A9C9E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26160" yWindow="5760" windowWidth="27640" windowHeight="16680" xr2:uid="{2CC304E0-977A-F44C-9ED5-57AAFC62DE41}"/>
+    <workbookView xWindow="0" yWindow="1000" windowWidth="34200" windowHeight="21000" xr2:uid="{2CC304E0-977A-F44C-9ED5-57AAFC62DE41}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="cannon" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -34,12 +34,125 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+  <si>
+    <t>Level</t>
+  </si>
+  <si>
+    <t>Hitpoints</t>
+  </si>
+  <si>
+    <t>Build Cost</t>
+  </si>
+  <si>
+    <t>5s</t>
+  </si>
+  <si>
+    <t>30s</t>
+  </si>
+  <si>
+    <t>2m</t>
+  </si>
+  <si>
+    <t>20m</t>
+  </si>
+  <si>
+    <t>30m</t>
+  </si>
+  <si>
+    <t>1h</t>
+  </si>
+  <si>
+    <t>2h</t>
+  </si>
+  <si>
+    <t>3h</t>
+  </si>
+  <si>
+    <t>3h 30m</t>
+  </si>
+  <si>
+    <t>4h</t>
+  </si>
+  <si>
+    <t>4h 30m</t>
+  </si>
+  <si>
+    <t>5h</t>
+  </si>
+  <si>
+    <t>6h</t>
+  </si>
+  <si>
+    <t>8h</t>
+  </si>
+  <si>
+    <t>10h</t>
+  </si>
+  <si>
+    <t>11h</t>
+  </si>
+  <si>
+    <t>12h</t>
+  </si>
+  <si>
+    <t>16h</t>
+  </si>
+  <si>
+    <t>20h</t>
+  </si>
+  <si>
+    <t>1d</t>
+  </si>
+  <si>
+    <t>1d 12h</t>
+  </si>
+  <si>
+    <t>DPSec</t>
+  </si>
+  <si>
+    <t>DPShot</t>
+  </si>
+  <si>
+    <t>Build time</t>
+  </si>
+  <si>
+    <t>Exp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TH Required </t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF3A3A3A"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="16"/>
+      <color rgb="FF3A3A3A"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="12"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -62,13 +175,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -381,9 +501,596 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CBDC0AC2-6795-D34F-B3EF-6458DFDE8454}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <dimension ref="A1:H23"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="16" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="16" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="5"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+    </row>
+    <row r="3" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>1</v>
+      </c>
+      <c r="B3" s="2">
+        <v>7</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5.6</v>
+      </c>
+      <c r="D3" s="2">
+        <v>300</v>
+      </c>
+      <c r="E3" s="2">
+        <v>250</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="G3" s="2">
+        <v>2</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>2</v>
+      </c>
+      <c r="B4" s="2">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2">
+        <v>8</v>
+      </c>
+      <c r="D4" s="2">
+        <v>360</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1000</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="2">
+        <v>5</v>
+      </c>
+      <c r="H4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>3</v>
+      </c>
+      <c r="B5" s="2">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2">
+        <v>10.4</v>
+      </c>
+      <c r="D5" s="2">
+        <v>420</v>
+      </c>
+      <c r="E5" s="3">
+        <v>4000</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G5" s="2">
+        <v>10</v>
+      </c>
+      <c r="H5" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>4</v>
+      </c>
+      <c r="B6" s="2">
+        <v>17</v>
+      </c>
+      <c r="C6" s="2">
+        <v>13.6</v>
+      </c>
+      <c r="D6" s="2">
+        <v>500</v>
+      </c>
+      <c r="E6" s="3">
+        <v>16000</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="G6" s="2">
+        <v>34</v>
+      </c>
+      <c r="H6" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2">
+        <v>23</v>
+      </c>
+      <c r="C7" s="2">
+        <v>18.399999999999999</v>
+      </c>
+      <c r="D7" s="2">
+        <v>600</v>
+      </c>
+      <c r="E7" s="3">
+        <v>50000</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="2">
+        <v>42</v>
+      </c>
+      <c r="H7" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2">
+        <v>30</v>
+      </c>
+      <c r="C8" s="2">
+        <v>24</v>
+      </c>
+      <c r="D8" s="2">
+        <v>660</v>
+      </c>
+      <c r="E8" s="3">
+        <v>60000</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G8" s="2">
+        <v>60</v>
+      </c>
+      <c r="H8" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2">
+        <v>40</v>
+      </c>
+      <c r="C9" s="2">
+        <v>32</v>
+      </c>
+      <c r="D9" s="2">
+        <v>730</v>
+      </c>
+      <c r="E9" s="3">
+        <v>100000</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G9" s="2">
+        <v>84</v>
+      </c>
+      <c r="H9" s="2">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>8</v>
+      </c>
+      <c r="B10" s="2">
+        <v>48</v>
+      </c>
+      <c r="C10" s="2">
+        <v>38.4</v>
+      </c>
+      <c r="D10" s="2">
+        <v>800</v>
+      </c>
+      <c r="E10" s="3">
+        <v>160000</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G10" s="2">
+        <v>103</v>
+      </c>
+      <c r="H10" s="2">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>9</v>
+      </c>
+      <c r="B11" s="2">
+        <v>56</v>
+      </c>
+      <c r="C11" s="2">
+        <v>44.8</v>
+      </c>
+      <c r="D11" s="2">
+        <v>880</v>
+      </c>
+      <c r="E11" s="3">
+        <v>250000</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="2">
+        <v>112</v>
+      </c>
+      <c r="H11" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>10</v>
+      </c>
+      <c r="B12" s="2">
+        <v>64</v>
+      </c>
+      <c r="C12" s="2">
+        <v>51.2</v>
+      </c>
+      <c r="D12" s="2">
+        <v>960</v>
+      </c>
+      <c r="E12" s="3">
+        <v>330000</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="2">
+        <v>120</v>
+      </c>
+      <c r="H12" s="2">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>11</v>
+      </c>
+      <c r="B13" s="2">
+        <v>74</v>
+      </c>
+      <c r="C13" s="2">
+        <v>59.2</v>
+      </c>
+      <c r="D13" s="3">
+        <v>1060</v>
+      </c>
+      <c r="E13" s="3">
+        <v>500000</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G13" s="2">
+        <v>127</v>
+      </c>
+      <c r="H13" s="1">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>12</v>
+      </c>
+      <c r="B14" s="2">
+        <v>85</v>
+      </c>
+      <c r="C14" s="2">
+        <v>68</v>
+      </c>
+      <c r="D14" s="3">
+        <v>1160</v>
+      </c>
+      <c r="E14" s="3">
+        <v>600000</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G14" s="2">
+        <v>134</v>
+      </c>
+      <c r="H14" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>13</v>
+      </c>
+      <c r="B15" s="2">
+        <v>95</v>
+      </c>
+      <c r="C15" s="2">
+        <v>76</v>
+      </c>
+      <c r="D15" s="3">
+        <v>1260</v>
+      </c>
+      <c r="E15" s="3">
+        <v>660000</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="G15" s="2">
+        <v>146</v>
+      </c>
+      <c r="H15" s="2">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>14</v>
+      </c>
+      <c r="B16" s="2">
+        <v>100</v>
+      </c>
+      <c r="C16" s="2">
+        <v>80</v>
+      </c>
+      <c r="D16" s="3">
+        <v>1380</v>
+      </c>
+      <c r="E16" s="3">
+        <v>1000000</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="2">
+        <v>169</v>
+      </c>
+      <c r="H16" s="1">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>15</v>
+      </c>
+      <c r="B17" s="2">
+        <v>105</v>
+      </c>
+      <c r="C17" s="2">
+        <v>84</v>
+      </c>
+      <c r="D17" s="3">
+        <v>1500</v>
+      </c>
+      <c r="E17" s="3">
+        <v>1200000</v>
+      </c>
+      <c r="F17" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="2">
+        <v>189</v>
+      </c>
+      <c r="H17" s="2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>16</v>
+      </c>
+      <c r="B18" s="2">
+        <v>110</v>
+      </c>
+      <c r="C18" s="2">
+        <v>88</v>
+      </c>
+      <c r="D18" s="3">
+        <v>1620</v>
+      </c>
+      <c r="E18" s="3">
+        <v>1300000</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G18" s="2">
+        <v>198</v>
+      </c>
+      <c r="H18" s="1">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>17</v>
+      </c>
+      <c r="B19" s="2">
+        <v>115</v>
+      </c>
+      <c r="C19" s="2">
+        <v>92</v>
+      </c>
+      <c r="D19" s="3">
+        <v>1740</v>
+      </c>
+      <c r="E19" s="3">
+        <v>1500000</v>
+      </c>
+      <c r="F19" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="2">
+        <v>207</v>
+      </c>
+      <c r="H19" s="2">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>18</v>
+      </c>
+      <c r="B20" s="2">
+        <v>125</v>
+      </c>
+      <c r="C20" s="2">
+        <v>100</v>
+      </c>
+      <c r="D20" s="3">
+        <v>1870</v>
+      </c>
+      <c r="E20" s="3">
+        <v>1800000</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" s="2">
+        <v>240</v>
+      </c>
+      <c r="H20" s="1">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>19</v>
+      </c>
+      <c r="B21" s="2">
+        <v>135</v>
+      </c>
+      <c r="C21" s="2">
+        <v>108</v>
+      </c>
+      <c r="D21" s="3">
+        <v>2000</v>
+      </c>
+      <c r="E21" s="3">
+        <v>2000000</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G21" s="2">
+        <v>268</v>
+      </c>
+      <c r="H21" s="2">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>20</v>
+      </c>
+      <c r="B22" s="2">
+        <v>150</v>
+      </c>
+      <c r="C22" s="2">
+        <v>120</v>
+      </c>
+      <c r="D22" s="3">
+        <v>2150</v>
+      </c>
+      <c r="E22" s="3">
+        <v>2600000</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="G22" s="2">
+        <v>293</v>
+      </c>
+      <c r="H22" s="1">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="21" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2">
+        <v>160</v>
+      </c>
+      <c r="C23" s="2">
+        <v>128</v>
+      </c>
+      <c r="D23" s="3">
+        <v>2250</v>
+      </c>
+      <c r="E23" s="3">
+        <v>3000000</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G23" s="2">
+        <v>360</v>
+      </c>
+      <c r="H23" s="2">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="G1" r:id="rId1" tooltip="Experience" display="https://clashofclans.fandom.com/wiki/Experience" xr:uid="{81AC77CC-8D9F-3444-A070-BFE353463024}"/>
+    <hyperlink ref="H1" r:id="rId2" tooltip="Town Hall" display="https://clashofclans.fandom.com/wiki/Town_Hall" xr:uid="{7511E465-37B2-DE4A-BD60-F300EA3E2999}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>